<commit_message>
updated test data for date implementation
</commit_message>
<xml_diff>
--- a/rules/CORE-000711/negative/01/data/unit-test-coreid-FB3404-negative.xlsx
+++ b/rules/CORE-000711/negative/01/data/unit-test-coreid-FB3404-negative.xlsx
@@ -53,6 +53,10 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
       <color rgb="FF000000"/>
     </font>
     <font>
@@ -75,13 +79,8 @@
       <name val="Calibri"/>
       <color rgb="FF000000"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <color rgb="FF000000"/>
-    </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -101,12 +100,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFCC"/>
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -148,11 +141,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -484,7 +477,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B2"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="str">
@@ -495,24 +488,16 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="4" t="str">
         <v>sdtmig</v>
       </c>
-      <c r="B2" s="4" t="str">
+      <c r="B2" s="5" t="str">
         <v>3-4</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="str">
-        <v/>
-      </c>
-      <c r="B3" s="4" t="str">
-        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -530,10 +515,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="4" t="str">
         <v>dm.xpt</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>Demographics</v>
       </c>
     </row>
@@ -569,122 +554,122 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2">
+      <c r="A2" s="4">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>dm.xpt</v>
       </c>
-      <c r="C2" s="2" t="str">
+      <c r="C2" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="4">
         <v>5</v>
       </c>
-      <c r="E2" s="2" t="str">
+      <c r="E2" s="4" t="str">
         <v>RFSTDTC</v>
       </c>
-      <c r="F2" s="2" t="str">
-        <v>2018-09-11</v>
+      <c r="F2" s="4" t="str">
+        <v>2018-08-04T11:00</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2">
+      <c r="A3" s="4">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="str">
+      <c r="B3" s="4" t="str">
         <v>dm.xpt</v>
       </c>
-      <c r="C3" s="2" t="str">
+      <c r="C3" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="4">
         <v>5</v>
       </c>
-      <c r="E3" s="2" t="str">
+      <c r="E3" s="4" t="str">
         <v>RFENDTC</v>
       </c>
-      <c r="F3" s="2" t="str">
+      <c r="F3" s="4" t="str">
         <v>2018-08-03</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2">
+      <c r="A4" s="4">
         <v>2</v>
       </c>
-      <c r="B4" s="2" t="str">
+      <c r="B4" s="4" t="str">
         <v>dm.xpt</v>
       </c>
-      <c r="C4" s="2" t="str">
+      <c r="C4" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="4">
         <v>6</v>
       </c>
-      <c r="E4" s="2" t="str">
+      <c r="E4" s="4" t="str">
         <v>RFSTDTC</v>
       </c>
-      <c r="F4" s="2" t="str">
+      <c r="F4" s="4" t="str">
+        <v>2018-11-06T12:01</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4">
+        <v>2</v>
+      </c>
+      <c r="B5" s="4" t="str">
+        <v>dm.xpt</v>
+      </c>
+      <c r="C5" s="4" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D5" s="4">
+        <v>6</v>
+      </c>
+      <c r="E5" s="4" t="str">
+        <v>RFENDTC</v>
+      </c>
+      <c r="F5" s="4" t="str">
         <v>2018-11-06T12:00</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2">
-        <v>2</v>
-      </c>
-      <c r="B5" s="2" t="str">
+    <row r="6">
+      <c r="A6" s="4">
+        <v>3</v>
+      </c>
+      <c r="B6" s="4" t="str">
         <v>dm.xpt</v>
       </c>
-      <c r="C5" s="2" t="str">
+      <c r="C6" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D5" s="2">
-        <v>6</v>
-      </c>
-      <c r="E5" s="2" t="str">
+      <c r="D6" s="4">
+        <v>7</v>
+      </c>
+      <c r="E6" s="4" t="str">
+        <v>RFSTDTC</v>
+      </c>
+      <c r="F6" s="4" t="str">
+        <v>2006-03</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4">
+        <v>3</v>
+      </c>
+      <c r="B7" s="4" t="str">
+        <v>dm.xpt</v>
+      </c>
+      <c r="C7" s="4" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D7" s="4">
+        <v>7</v>
+      </c>
+      <c r="E7" s="4" t="str">
         <v>RFENDTC</v>
       </c>
-      <c r="F5" s="2" t="str">
-        <v>2018-11-06</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2">
-        <v>3</v>
-      </c>
-      <c r="B6" s="2" t="str">
-        <v>dm.xpt</v>
-      </c>
-      <c r="C6" s="2" t="str">
-        <v>Record</v>
-      </c>
-      <c r="D6" s="2">
-        <v>7</v>
-      </c>
-      <c r="E6" s="2" t="str">
-        <v>RFSTDTC</v>
-      </c>
-      <c r="F6" s="2" t="str">
-        <v>2006-03</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2">
-        <v>3</v>
-      </c>
-      <c r="B7" s="2" t="str">
-        <v>dm.xpt</v>
-      </c>
-      <c r="C7" s="2" t="str">
-        <v>Record</v>
-      </c>
-      <c r="D7" s="2">
-        <v>7</v>
-      </c>
-      <c r="E7" s="2" t="str">
-        <v>RFENDTC</v>
-      </c>
-      <c r="F7" s="2" t="str">
+      <c r="F7" s="4" t="str">
         <v>2006-01-16</v>
       </c>
     </row>
@@ -780,642 +765,642 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="str">
+      <c r="A2" s="6" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="5" t="str">
+      <c r="B2" s="6" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="6" t="str">
+      <c r="C2" s="7" t="str">
         <v>Unique Subject Identifier</v>
       </c>
-      <c r="D2" s="6" t="str">
+      <c r="D2" s="7" t="str">
         <v>Subject Identifier for the Study</v>
       </c>
-      <c r="E2" s="6" t="str">
+      <c r="E2" s="7" t="str">
         <v>Subject Reference Start Date/Time</v>
       </c>
-      <c r="F2" s="6" t="str">
+      <c r="F2" s="7" t="str">
         <v>Subject Reference End Date/Time</v>
       </c>
-      <c r="G2" s="6" t="str">
+      <c r="G2" s="7" t="str">
         <v>Date/Time of First Study Treatment</v>
       </c>
-      <c r="H2" s="6" t="str">
+      <c r="H2" s="7" t="str">
         <v>Date/Time of Last Study Treatment</v>
       </c>
-      <c r="I2" s="6" t="str">
+      <c r="I2" s="7" t="str">
         <v>Date/Time of Informed Consent</v>
       </c>
-      <c r="J2" s="6" t="str">
+      <c r="J2" s="7" t="str">
         <v>Date/Time of End of Participation</v>
       </c>
-      <c r="K2" s="6" t="str">
+      <c r="K2" s="7" t="str">
         <v>Date/Time of Death</v>
       </c>
-      <c r="L2" s="6" t="str">
+      <c r="L2" s="7" t="str">
         <v>Subject Death Flag</v>
       </c>
-      <c r="M2" s="6" t="str">
+      <c r="M2" s="7" t="str">
         <v>Study Site Identifier</v>
       </c>
-      <c r="N2" s="6" t="str">
+      <c r="N2" s="7" t="str">
         <v>Date/Time of Birth</v>
       </c>
-      <c r="O2" s="6" t="str">
+      <c r="O2" s="7" t="str">
         <v>Age</v>
       </c>
-      <c r="P2" s="6" t="str">
+      <c r="P2" s="7" t="str">
         <v>Age Units</v>
       </c>
-      <c r="Q2" s="6" t="str">
+      <c r="Q2" s="7" t="str">
         <v>Sex</v>
       </c>
-      <c r="R2" s="6" t="str">
+      <c r="R2" s="7" t="str">
         <v>Race</v>
       </c>
-      <c r="S2" s="6" t="str">
+      <c r="S2" s="7" t="str">
         <v>Ethnicity</v>
       </c>
-      <c r="T2" s="6" t="str">
+      <c r="T2" s="7" t="str">
         <v>Planned Arm Code</v>
       </c>
-      <c r="U2" s="6" t="str">
+      <c r="U2" s="7" t="str">
         <v>Description of Planned Arm</v>
       </c>
-      <c r="V2" s="6" t="str">
+      <c r="V2" s="7" t="str">
         <v>Actual Arm Code</v>
       </c>
-      <c r="W2" s="6" t="str">
+      <c r="W2" s="7" t="str">
         <v>Description of Actual Arm</v>
       </c>
-      <c r="X2" s="6" t="str">
+      <c r="X2" s="7" t="str">
         <v>Reason Arm and/or Actual Arm is Null</v>
       </c>
-      <c r="Y2" s="6" t="str">
+      <c r="Y2" s="7" t="str">
         <v>Description of Unplanned Actual Arm</v>
       </c>
-      <c r="Z2" s="6" t="str">
+      <c r="Z2" s="7" t="str">
         <v>Country</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="B3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="C3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="D3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="E3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="F3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="G3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="H3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="I3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="J3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="K3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="L3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="M3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="N3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="O3" s="6" t="str">
+      <c r="A3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="D3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="E3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="F3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="G3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="H3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="I3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="J3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="K3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="L3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="M3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="N3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="O3" s="7" t="str">
         <v>Num</v>
       </c>
-      <c r="P3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="Q3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="R3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="S3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="T3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="U3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="V3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="W3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="X3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="Y3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="Z3" s="6" t="str">
+      <c r="P3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="Q3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="R3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="S3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="T3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="U3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="V3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="W3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="X3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="Y3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="Z3" s="7" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6">
+      <c r="A4" s="7">
         <v>12</v>
       </c>
-      <c r="B4" s="6">
+      <c r="B4" s="7">
         <v>2</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="7">
         <v>8</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="7">
         <v>4</v>
       </c>
-      <c r="E4" s="6" t="str">
+      <c r="E4" s="7" t="str">
         <v>19</v>
       </c>
-      <c r="F4" s="6" t="str">
+      <c r="F4" s="7" t="str">
         <v>19</v>
       </c>
-      <c r="G4" s="6" t="str">
+      <c r="G4" s="7" t="str">
         <v>19</v>
       </c>
-      <c r="H4" s="6" t="str">
+      <c r="H4" s="7" t="str">
         <v>19</v>
       </c>
-      <c r="I4" s="6" t="str">
+      <c r="I4" s="7" t="str">
         <v>19</v>
       </c>
-      <c r="J4" s="6" t="str">
+      <c r="J4" s="7" t="str">
         <v>19</v>
       </c>
-      <c r="K4" s="6" t="str">
+      <c r="K4" s="7" t="str">
         <v>19</v>
       </c>
-      <c r="L4" s="6">
+      <c r="L4" s="7">
         <v>1</v>
       </c>
-      <c r="M4" s="6">
+      <c r="M4" s="7">
         <v>3</v>
       </c>
-      <c r="N4" s="6" t="str">
+      <c r="N4" s="7" t="str">
         <v>19</v>
       </c>
-      <c r="O4" s="6">
+      <c r="O4" s="7">
         <v>8</v>
       </c>
-      <c r="P4" s="6">
+      <c r="P4" s="7">
         <v>5</v>
       </c>
-      <c r="Q4" s="6">
+      <c r="Q4" s="7">
         <v>1</v>
       </c>
-      <c r="R4" s="6">
+      <c r="R4" s="7">
         <v>41</v>
       </c>
-      <c r="S4" s="6">
+      <c r="S4" s="7">
         <v>22</v>
       </c>
-      <c r="T4" s="6">
+      <c r="T4" s="7">
         <v>8</v>
       </c>
-      <c r="U4" s="6">
+      <c r="U4" s="7">
         <v>28</v>
       </c>
-      <c r="V4" s="6">
+      <c r="V4" s="7">
         <v>8</v>
       </c>
-      <c r="W4" s="6">
+      <c r="W4" s="7">
         <v>28</v>
       </c>
-      <c r="X4" s="6">
+      <c r="X4" s="7">
         <v>14</v>
       </c>
-      <c r="Y4" s="6">
+      <c r="Y4" s="7">
         <v>200</v>
       </c>
-      <c r="Z4" s="6">
+      <c r="Z4" s="7">
         <v>3</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="str">
+      <c r="A5" s="5" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B5" s="4" t="str">
+      <c r="B5" s="5" t="str">
         <v>DM</v>
       </c>
-      <c r="C5" s="4" t="str">
+      <c r="C5" s="5" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="5">
         <v>1115</v>
       </c>
-      <c r="E5" s="7" t="str">
-        <v>2018-09-11</v>
+      <c r="E5" s="8" t="str">
+        <v>2018-08-04T11:00</v>
       </c>
       <c r="F5" s="8" t="str">
         <v>2018-08-03</v>
       </c>
-      <c r="G5" s="4" t="str">
+      <c r="G5" s="5" t="str">
         <v>2018-05-17T09:35</v>
       </c>
-      <c r="H5" s="4" t="str">
+      <c r="H5" s="5" t="str">
         <v>2018-08-03</v>
       </c>
-      <c r="I5" s="4" t="str">
+      <c r="I5" s="5" t="str">
         <v>2018-04-26</v>
       </c>
-      <c r="J5" s="4" t="str">
+      <c r="J5" s="5" t="str">
         <v>2018-08-22</v>
       </c>
-      <c r="K5" s="4" t="str">
+      <c r="K5" s="5" t="str">
         <v>2018-08-22</v>
       </c>
-      <c r="L5" s="4" t="str">
+      <c r="L5" s="5" t="str">
         <v>Y</v>
       </c>
-      <c r="M5" s="4">
+      <c r="M5" s="5">
         <v>701</v>
       </c>
-      <c r="N5" s="4" t="str">
+      <c r="N5" s="5" t="str">
         <v>1947-07-24</v>
       </c>
-      <c r="O5" s="4" t="str">
+      <c r="O5" s="5" t="str">
         <v>70</v>
       </c>
-      <c r="P5" s="4" t="str">
+      <c r="P5" s="5" t="str">
         <v>YEARS</v>
       </c>
-      <c r="Q5" s="4" t="str">
+      <c r="Q5" s="5" t="str">
         <v>M</v>
       </c>
-      <c r="R5" s="4" t="str">
+      <c r="R5" s="5" t="str">
         <v>WHITE</v>
       </c>
-      <c r="S5" s="4" t="str">
+      <c r="S5" s="5" t="str">
         <v>NOT HISPANIC OR LATINO</v>
       </c>
-      <c r="T5" s="4" t="str">
+      <c r="T5" s="5" t="str">
         <v>A</v>
       </c>
-      <c r="U5" s="4" t="str">
+      <c r="U5" s="5" t="str">
         <v>Drug A</v>
       </c>
-      <c r="V5" s="4" t="str">
+      <c r="V5" s="5" t="str">
         <v>A</v>
       </c>
-      <c r="W5" s="4" t="str">
+      <c r="W5" s="5" t="str">
         <v>Drug A</v>
       </c>
-      <c r="X5" s="4" t="str">
+      <c r="X5" s="5" t="str">
         <v/>
       </c>
-      <c r="Y5" s="4" t="str">
+      <c r="Y5" s="5" t="str">
         <v/>
       </c>
-      <c r="Z5" s="4" t="str">
+      <c r="Z5" s="5" t="str">
         <v>AUS</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="str">
+      <c r="A6" s="5" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B6" s="4" t="str">
+      <c r="B6" s="5" t="str">
         <v>DM</v>
       </c>
-      <c r="C6" s="4" t="str">
+      <c r="C6" s="5" t="str">
         <v>CDISC002</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="5">
         <v>1211</v>
       </c>
-      <c r="E6" s="7" t="str">
+      <c r="E6" s="9" t="str">
+        <v>2018-11-06T12:01</v>
+      </c>
+      <c r="F6" s="9" t="str">
         <v>2018-11-06T12:00</v>
       </c>
-      <c r="F6" s="8" t="str">
+      <c r="G6" s="5" t="str">
+        <v>2018-05-24T12:00</v>
+      </c>
+      <c r="H6" s="5" t="str">
         <v>2018-11-06</v>
       </c>
-      <c r="G6" s="4" t="str">
-        <v>2018-05-24T12:00</v>
-      </c>
-      <c r="H6" s="4" t="str">
-        <v>2018-11-06</v>
-      </c>
-      <c r="I6" s="4" t="str">
+      <c r="I6" s="5" t="str">
         <v>2018-05-07</v>
       </c>
-      <c r="J6" s="4" t="str">
+      <c r="J6" s="5" t="str">
         <v>2019-02-04</v>
       </c>
-      <c r="K6" s="4" t="str">
+      <c r="K6" s="5" t="str">
         <v>2019-02-04</v>
       </c>
-      <c r="L6" s="4" t="str">
+      <c r="L6" s="5" t="str">
         <v>Y</v>
       </c>
-      <c r="M6" s="4">
+      <c r="M6" s="5">
         <v>701</v>
       </c>
-      <c r="N6" s="4" t="str">
+      <c r="N6" s="5" t="str">
         <v>1905-05-08</v>
       </c>
-      <c r="O6" s="4" t="str">
+      <c r="O6" s="5" t="str">
         <v>78</v>
       </c>
-      <c r="P6" s="4" t="str">
+      <c r="P6" s="5" t="str">
         <v>YEARS</v>
       </c>
-      <c r="Q6" s="4" t="str">
+      <c r="Q6" s="5" t="str">
         <v>M</v>
       </c>
-      <c r="R6" s="4" t="str">
+      <c r="R6" s="5" t="str">
         <v>WHITE</v>
       </c>
-      <c r="S6" s="4" t="str">
+      <c r="S6" s="5" t="str">
         <v>NOT HISPANIC OR LATINO</v>
       </c>
-      <c r="T6" s="4" t="str">
+      <c r="T6" s="5" t="str">
         <v>P</v>
       </c>
-      <c r="U6" s="4" t="str">
+      <c r="U6" s="5" t="str">
         <v>Placebo</v>
       </c>
-      <c r="V6" s="4" t="str">
+      <c r="V6" s="5" t="str">
         <v>P</v>
       </c>
-      <c r="W6" s="4" t="str">
+      <c r="W6" s="5" t="str">
         <v>Placebo</v>
       </c>
-      <c r="X6" s="4" t="str">
+      <c r="X6" s="5" t="str">
         <v/>
       </c>
-      <c r="Y6" s="4" t="str">
+      <c r="Y6" s="5" t="str">
         <v/>
       </c>
-      <c r="Z6" s="4" t="str">
+      <c r="Z6" s="5" t="str">
         <v>AUS</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="str">
+      <c r="A7" s="5" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B7" s="4" t="str">
+      <c r="B7" s="5" t="str">
         <v>DM</v>
       </c>
-      <c r="C7" s="4" t="str">
+      <c r="C7" s="5" t="str">
         <v>CDISC003</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D7" s="5">
         <v>1302</v>
       </c>
       <c r="E7" s="9" t="str">
         <v>2006-03</v>
       </c>
-      <c r="F7" s="8" t="str">
+      <c r="F7" s="9" t="str">
         <v>2006-01-16</v>
       </c>
-      <c r="G7" s="4" t="str">
+      <c r="G7" s="5" t="str">
         <v>2006-01-16</v>
       </c>
-      <c r="H7" s="4" t="str">
+      <c r="H7" s="5" t="str">
         <v>2006-03-19</v>
       </c>
-      <c r="I7" s="4" t="str">
+      <c r="I7" s="5" t="str">
         <v>2006-01-02</v>
       </c>
-      <c r="J7" s="4" t="str">
+      <c r="J7" s="5" t="str">
         <v>2006-03-19</v>
       </c>
-      <c r="K7" s="4" t="str">
+      <c r="K7" s="5" t="str">
         <v>2018-12-11</v>
       </c>
-      <c r="L7" s="4" t="str">
+      <c r="L7" s="5" t="str">
         <v>Y</v>
       </c>
-      <c r="M7" s="4">
+      <c r="M7" s="5">
         <v>701</v>
       </c>
-      <c r="N7" s="4" t="str">
+      <c r="N7" s="5" t="str">
         <v>1944-06-16</v>
       </c>
-      <c r="O7" s="4" t="str">
+      <c r="O7" s="5" t="str">
         <v>74</v>
       </c>
-      <c r="P7" s="4" t="str">
+      <c r="P7" s="5" t="str">
         <v>YEARS</v>
       </c>
-      <c r="Q7" s="4" t="str">
+      <c r="Q7" s="5" t="str">
         <v>M</v>
       </c>
-      <c r="R7" s="4" t="str">
+      <c r="R7" s="5" t="str">
         <v>WHITE</v>
       </c>
-      <c r="S7" s="4" t="str">
+      <c r="S7" s="5" t="str">
         <v>NOT HISPANIC OR LATINO</v>
       </c>
-      <c r="T7" s="4" t="str">
+      <c r="T7" s="5" t="str">
         <v>B</v>
       </c>
-      <c r="U7" s="4" t="str">
+      <c r="U7" s="5" t="str">
         <v>Drug B</v>
       </c>
-      <c r="V7" s="4" t="str">
+      <c r="V7" s="5" t="str">
         <v>B</v>
       </c>
-      <c r="W7" s="4" t="str">
+      <c r="W7" s="5" t="str">
         <v>Drug B</v>
       </c>
-      <c r="X7" s="4" t="str">
+      <c r="X7" s="5" t="str">
         <v/>
       </c>
-      <c r="Y7" s="4" t="str">
+      <c r="Y7" s="5" t="str">
         <v/>
       </c>
-      <c r="Z7" s="4" t="str">
+      <c r="Z7" s="5" t="str">
         <v>CZE</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="str">
+      <c r="A8" s="5" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B8" s="4" t="str">
+      <c r="B8" s="5" t="str">
         <v>DM</v>
       </c>
-      <c r="C8" s="4" t="str">
+      <c r="C8" s="5" t="str">
         <v>CDISC004</v>
       </c>
-      <c r="D8" s="4">
+      <c r="D8" s="5">
         <v>1402</v>
       </c>
-      <c r="E8" s="4" t="str">
+      <c r="E8" s="5" t="str">
         <v>2018-07-16T09:15</v>
       </c>
-      <c r="F8" s="4" t="str">
+      <c r="F8" s="5" t="str">
         <v>2018-11-06T14:00</v>
       </c>
-      <c r="G8" s="4" t="str">
+      <c r="G8" s="5" t="str">
         <v>2018-07-16T09:15</v>
       </c>
-      <c r="H8" s="4" t="str">
+      <c r="H8" s="5" t="str">
         <v>2018-11-06T14:00</v>
       </c>
-      <c r="I8" s="4" t="str">
+      <c r="I8" s="5" t="str">
         <v>2018-06-27</v>
       </c>
-      <c r="J8" s="4" t="str">
+      <c r="J8" s="5" t="str">
         <v>2018-12-11</v>
       </c>
-      <c r="K8" s="2" t="str">
+      <c r="K8" s="4" t="str">
         <v/>
       </c>
-      <c r="L8" s="2" t="str">
+      <c r="L8" s="4" t="str">
         <v/>
       </c>
-      <c r="M8" s="4">
+      <c r="M8" s="5">
         <v>701</v>
       </c>
-      <c r="N8" s="4" t="str">
+      <c r="N8" s="5" t="str">
         <v>1905-04-16</v>
       </c>
-      <c r="O8" s="4" t="str">
+      <c r="O8" s="5" t="str">
         <v>68</v>
       </c>
-      <c r="P8" s="4" t="str">
+      <c r="P8" s="5" t="str">
         <v>YEARS</v>
       </c>
-      <c r="Q8" s="4" t="str">
+      <c r="Q8" s="5" t="str">
         <v>F</v>
       </c>
-      <c r="R8" s="4" t="str">
+      <c r="R8" s="5" t="str">
         <v>WHITE</v>
       </c>
-      <c r="S8" s="4" t="str">
+      <c r="S8" s="5" t="str">
         <v>HISPANIC OR LATINO</v>
       </c>
-      <c r="T8" s="4" t="str">
+      <c r="T8" s="5" t="str">
         <v>B</v>
       </c>
-      <c r="U8" s="4" t="str">
+      <c r="U8" s="5" t="str">
         <v>Drug B</v>
       </c>
-      <c r="V8" s="4" t="str">
+      <c r="V8" s="5" t="str">
         <v>B</v>
       </c>
-      <c r="W8" s="4" t="str">
+      <c r="W8" s="5" t="str">
         <v>Drug B</v>
       </c>
-      <c r="X8" s="4" t="str">
+      <c r="X8" s="5" t="str">
         <v/>
       </c>
-      <c r="Y8" s="4" t="str">
+      <c r="Y8" s="5" t="str">
         <v/>
       </c>
-      <c r="Z8" s="4" t="str">
+      <c r="Z8" s="5" t="str">
         <v>CAN</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="str">
+      <c r="A9" s="5" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B9" s="4" t="str">
+      <c r="B9" s="5" t="str">
         <v>DM</v>
       </c>
-      <c r="C9" s="4" t="str">
+      <c r="C9" s="5" t="str">
         <v>CDISC005</v>
       </c>
-      <c r="D9" s="4">
+      <c r="D9" s="5">
         <v>1502</v>
       </c>
-      <c r="E9" s="4" t="str">
+      <c r="E9" s="5" t="str">
         <v>2006</v>
       </c>
-      <c r="F9" s="4" t="str">
+      <c r="F9" s="5" t="str">
         <v>2006-01-16</v>
       </c>
-      <c r="G9" s="4" t="str">
+      <c r="G9" s="5" t="str">
         <v>2006-01-16</v>
       </c>
-      <c r="H9" s="4" t="str">
+      <c r="H9" s="5" t="str">
         <v>2006-03-19</v>
       </c>
-      <c r="I9" s="4" t="str">
+      <c r="I9" s="5" t="str">
         <v>2006-01-02</v>
       </c>
-      <c r="J9" s="4" t="str">
+      <c r="J9" s="5" t="str">
         <v>2006-03-19</v>
       </c>
-      <c r="K9" s="4" t="str">
+      <c r="K9" s="5" t="str">
         <v>2018-12-11</v>
       </c>
-      <c r="L9" s="4" t="str">
+      <c r="L9" s="5" t="str">
         <v>Y</v>
       </c>
-      <c r="M9" s="4">
+      <c r="M9" s="5">
         <v>701</v>
       </c>
-      <c r="N9" s="4" t="str">
+      <c r="N9" s="5" t="str">
         <v>1944-06-16</v>
       </c>
-      <c r="O9" s="4" t="str">
+      <c r="O9" s="5" t="str">
         <v>74</v>
       </c>
-      <c r="P9" s="4" t="str">
+      <c r="P9" s="5" t="str">
         <v>YEARS</v>
       </c>
-      <c r="Q9" s="4" t="str">
+      <c r="Q9" s="5" t="str">
         <v>M</v>
       </c>
-      <c r="R9" s="4" t="str">
+      <c r="R9" s="5" t="str">
         <v>WHITE</v>
       </c>
-      <c r="S9" s="4" t="str">
+      <c r="S9" s="5" t="str">
         <v>NOT HISPANIC OR LATINO</v>
       </c>
-      <c r="T9" s="4" t="str">
+      <c r="T9" s="5" t="str">
         <v>B</v>
       </c>
-      <c r="U9" s="4" t="str">
+      <c r="U9" s="5" t="str">
         <v>Drug B</v>
       </c>
-      <c r="V9" s="4" t="str">
+      <c r="V9" s="5" t="str">
         <v>B</v>
       </c>
-      <c r="W9" s="4" t="str">
+      <c r="W9" s="5" t="str">
         <v>Drug B</v>
       </c>
-      <c r="X9" s="4" t="str">
+      <c r="X9" s="5" t="str">
         <v/>
       </c>
-      <c r="Y9" s="4" t="str">
+      <c r="Y9" s="5" t="str">
         <v/>
       </c>
-      <c r="Z9" s="4" t="str">
+      <c r="Z9" s="5" t="str">
         <v>CZE</v>
       </c>
     </row>

</xml_diff>